<commit_message>
audit(ledger): 2026-09-01 scrub — F97 closed live, F03 fixed, F73 blocked
F97 CLOSED LIVE: yesterday's eyebrow wrap verified on production at an
emulated 375x812 — flex-wrap wrap, 0px overflow, read-time visible, no
document overflow, article.css?v=phase37 serving the rule.

F03 opened and fixed this run (MEDIUM): the theme-color clause of its
expected behaviour had never been satisfiable. Fix + retest recorded.

F73 upgraded from suspicion to a confirmed pattern: five consecutive
hook-triggered deploys land +4h52m to +12h16m off the 05:05 UTC cron but
never miss a day — GitHub Actions queue latency, not repo config. Marked
BLOCKED; the only real remedy is outside the repo.

29 rows carry fresh live-verification notes. F35/F36 recorded as a rotation
gap (pane-hidden scroll, neither PASS nor FAIL). F75 source-verified only.
No rows added — the only commit since the last ledger write touched
DESIGN-SYSTEM.md alone.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/imjustdex-feature-audit.xlsx
+++ b/audit/imjustdex-feature-audit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Features" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$3:$K$100</definedName>
@@ -652,7 +652,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus.</t>
+          <t>PASS — masthead .brand-block → '/' present on home/about/404/phase0/brand/article; aria-label 'Dexter Jakes home' | 2026-08-15 re-verified live: brand-block present and linking / on all 20 pages | 2026-08-25 re-verified live: brand-block present and linking / on all 20 crawled routes; aria-label intact. | 2026-08-27 re-verified live: masthead .brand-block → '/' confirmed under real Tab focus. | 2026-09-01 re-verified live: masthead .brand-block reached under a REAL Tab press (2nd stop), links '/', focus ring #c00 2px.</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about.</t>
+          <t>PASS — brand-word: Words (home/article/about/brand), 404, Phase 0 — matches documented intent | 2026-08-15 re-verified live: brand-word: home/about/article 'Words', 404 '404', phase0 'Phase 0' — matches the documented about-page quirk | 2026-08-25 re-verified live: brand-word: "Words" on home/about/article, "404" on /404, "Phase 0" on /phase0/ — matches documented intent. | 2026-08-27 re-verified live: brand word 'Words' confirmed on home/article/about. | 2026-09-01 re-verified live on the homepage: masthead brand word reads 'Words' (documented intent). Other surfaces not re-walked this run.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -754,14 +754,22 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks.</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>PASS — toggle cycles dark→light→dark; dxmode cookie written both ways; label + aria-pressed + bg/ink all update. Reconfirmed 2026-08-10 PM across 3 consecutive clicks. | 2026-08-13 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways; --bg/--ink/--accent-text all re-resolved (#060606/#f3f0e8/#ff4d4d dark, #f4f4f1/#050505/#c00 light). | 2026-08-16 re-verified live: toggle cycled dark-&gt;light-&gt;dark on the live homepage; dxmode cookie written both ways (dxmode=light then dxmode=dark); --bg #060606&lt;-&gt;#f4f4f1 and --ink #f3f0e8&lt;-&gt;#050505 both re-resolved; label and aria-pressed tracked ('Mode: Dark'/true &lt;-&gt; 'Mode: Light'/false). | 2026-08-25 re-verified live: toggle re-verified with a REAL pointer click (not element.click()) on both the homepage and /words/the-stone/: page repaints dark&lt;-&gt;light, dxmode cookie written both ways, label and aria-pressed track. METHOD NOTE: a programmatic element.click() flips the class, the tokens and the cookie but leaves body's used background/color stale in getComputedStyle until a repaint is forced — that is a measurement artifact, NOT a site defect, and it read as an article-page mode regression for several minutes this run. Always verify this row with a real click. | 2026-08-27 re-verified live: REAL pointer click (not element.click()) + 2s settle + screenshot: dark→light→dark, --bg #060606↔#f4f4f1, --ink #f3f0e8↔#050505, dxmode cookie written both ways, button label tracks. | 2026-09-01 ISSUE (MEDIUM) — theme-color half of this row has NEVER been satisfiable. mode.js ships syncThemeColor() (js/mode.js:74-95) which rewrites &lt;meta name="theme-color"&gt; to #060606/#f4f4f1 and strips the media attr off a media-split pair, but NO layout ever emitted that meta: document.querySelectorAll('meta[name="theme-color"]').length === 0 on /, /about/, /words/&lt;slug&gt;/, /404, /brand/ and /phase0/ live. querySelector() returned null, the function no-opped, and the dedupe loop iterated an empty list — silent, so five months of scrubs that checked the class/cookie/tokens never saw it. User-visible effect: mobile browser chrome (address/status bar) follows the OS instead of the site's mode. Class flip, dxmode cookie, --bg/--ink re-resolve, aria-pressed, label and logo swap all re-verified live PASS this run with a REAL pointer click + 2s settle.</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM (fixed)</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | 2026-09-01 FIX: added the media-split pair mode.js was written to collapse — &lt;meta name="theme-color" content="#f4f4f1" media="(prefers-color-scheme: light)"&gt; + &lt;meta ... content="#060606" media="(prefers-color-scheme: dark)"&gt; — immediately after the existing &lt;meta name="color-scheme"&gt; in all 7 head sources: src/layouts/{Home,Article,ComingSoon}Layout.astro, src/pages/404.astro, src/pages/about.astro, brand/index.html, phase0/index.html. brand/ and public/brand/ (and phase0/) are HARDLINKS (verified same inode before and after the write), so the F87 dogfood contract is satisfied by a single edit each. Colours are not new design — they are the values already hardcoded in mode.js and equal to the --bg token in each mode. No cache-bust needed: only HTML changed, and HTML is served no-cache; mode.js is untouched at phase11.</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>PASS | 2026-09-01 RETEST (verified against local build of qa/fixes-20260901, npm run build clean, 20 pages): pre-JS HTML carries both media-split metas; after DOMContentLoaded mode.js collapses them to exactly ONE meta with the media attr stripped on every route type — / /about/ /404 /words/the-weight-of-my-no/ /brand/ /phase0/ all report count:1. Toggle dark -&gt; content #060606, cookie dxmode=dark; back to light -&gt; #f4f4f1, cookie dxmode=light. Zero console errors. Regression sanity: F97's eyebrow unaffected (flex-wrap nowrap + overflow 0 at desktop, as designed), single h1 intact on every retested route. Goes live-verified on the next SCRUB after Dexter merges.</t>
         </is>
       </c>
     </row>
@@ -803,7 +811,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive.</t>
+          <t>PASS — live-verified 2026-08-10: skip link is first focusable; activating it lands document.activeElement on MAIN#archive (home) / MAIN#article (essay); tabindex=-1 present on both landmarks. The 2c7d88d fix holds in production. | 2026-08-13 re-verified live: tab-target verified on live: .skip-link reveals from left:-999px to a 83x69 box at (12,12), cream-on-ink 17.79:1; activating it moved document.activeElement to MAIN#archive (tabindex=-1). Article pages target #article. | 2026-08-16 re-verified live: structural half re-verified live: .skip-link is the first focusable element in document order on every page type, and its target (MAIN#article / MAIN#archive / MAIN#phase0 / MAIN#main) carries tabindex=-1. End-to-end activation NOT re-exercisable this run — the browser pane reports document.visibilityState 'hidden' and drops page focus on every reload, so a fresh-load Tab lands on BODY. Harness limitation, not a site regression; last live activation was 2026-08-13. NOTE: this row's sweep is what surfaced F91 — see that row. | 2026-08-25 re-verified live: verified end-to-end live under REAL keyboard input on /words/the-stone/ — the gap the 2026-08-16 run had to leave open. .skip-link is the first focusable in DOM order, reveals from left:-999px to a 126x46 chip at (12,12), computes 17.79:1 (#060606 on #f3f0e8), and pressing Enter sets location.hash to #article and moves document.activeElement to MAIN#article (tabindex=-1). | 2026-08-27 re-verified live: skip link is the first focusable (reached by real shift+Tab from .brand-block), renders as an opaque cream chip at 17.79:1, and activation moves focus to MAIN#archive with hash #archive. | 2026-09-01 re-verified live: .skip-link is the FIRST Tab stop from page load and matches :focus-visible; activation moves location.hash to #archive and focus to MAIN#archive. Ran the ordinary-link control first per the harness antipattern.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -954,7 +962,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head.</t>
+          <t>PASS (2026-08-15 scrub) — home/about/phase0/articles all carry the feed discovery link; /404 correctly omits it. NOTE: the prior `expected` said articles do NOT include it. That text was stale — ArticleLayout has emitted the link since a4f4f25; the site was never wrong, the row was. Expectation corrected, not the code. | 2026-08-25 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head. | 2026-09-01 re-verified live: &lt;link rel=alternate type=application/atom+xml href=/feed.xml&gt; present in head; /feed.xml 200.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -1007,7 +1015,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200.</t>
+          <t>PASS — /img/favicon-32.png + /img/apple-touch-icon.png 200 on every referenced path | 2026-08-15 re-verified live: favicon-32.png + apple-touch-icon.png linked on every page; both 200 (1327b / 5729b) | 2026-08-25 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200 on every referenced path. | 2026-08-27 re-verified live: /img/favicon-32.png + /img/apple-touch-icon.png 200. | 2026-09-01 re-verified live: /img/favicon-32.png 200, /img/apple-touch-icon.png 200, /img/logo-dark.svg 200.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1056,7 +1064,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed.</t>
+          <t>PASS — Anton + IBM Plex Sans self-hosted, preloaded, document.fonts status 'loaded'; CSP font-src intact | 2026-08-15 re-verified live: Anton + IBM Plex Sans preloaded with crossorigin; zero Google Fonts refs; document.fonts reports all 3 faces loaded | 2026-08-16 re-verified live: Anton + IBM Plex Sans (Regular/Bold) all report document.fonts status 'loaded', document.fonts.status 'loaded'; zero Google Fonts references. /brand/ additionally preloads IBMPlexSans-Italic.woff2 and the console warns it is 'not used within a few seconds of load' — investigated and DISMISSED as a non-finding: the italic face is genuinely used by 13 elements on that page and reports status 'loaded'; the warning is a below-the-fold timing artifact. No other page preloads italic, which is correct. | 2026-08-25 re-verified live: document.fonts.status "loaded"; Anton/400, IBM Plex Sans/400 and /700 all report loaded. All three woff2 200. No FOUT observed. | 2026-08-27 re-verified live: document.fonts: Anton 400, IBM Plex Sans 400 + 700 all 'loaded'; fonts.status 'loaded'; no FOUT observed. | 2026-09-01 re-verified live via document.fonts (not the CSS stack): Anton 400 loaded, IBM Plex Sans 400 + 700 loaded; document.fonts.check() true for all three on home and article. No FOUT/FOIT observed.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1105,7 +1113,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages</t>
+          <t>PASS — no horizontal overflow at 390px on home/article/about/phase0/brand/404 | 2026-08-15 re-verified live: viewport width=device-width + viewport-fit=cover on all pages | 2026-09-01 re-verified live at an emulated 375x812: documentElement.scrollWidth == clientWidth == 375 on the article page — zero horizontal overflow.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1158,7 +1166,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes.</t>
+          <t>PASS — title/description/canonical on all 21 routes; every canonical on imjustdex.com | 2026-08-15 re-verified live: zero duplicate &lt;title&gt; across 20 pages; /404 canonical is /404 as specified | 2026-08-25 re-verified live: &lt;title&gt;, meta description and canonical present and correct on all 20 routes; every canonical points at imjustdex.com. | 2026-08-27 re-verified live: title/description/canonical present and on-domain across all 21 routes. | 2026-09-01 re-verified live: &lt;title&gt;, meta description and canonical present on all 17 articles plus / and /about/; canonicals all on imjustdex.com.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1207,7 +1215,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200.</t>
+          <t>PASS — og+twitter complete on all 21; all 19 OG images 200 (16 essays + home/about/phase0/brand) | 2026-08-15 re-verified live: twitter:card summary_large_image on every page in scope (404 correctly excluded) | 2026-08-25 re-verified live: og:title / og:description / og:image present on all 20; all 16 og-&lt;slug&gt;.png 200; og:image byte-identical to the JSON-LD image on all 16. | 2026-08-27 re-verified live: og+twitter complete across 21 routes; all 21 distinct OG images 200. | 2026-09-01 re-verified live: og:image resolves 200 on all 17 articles and every one matches the JSON-LD image URL exactly, cache-bust included.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1260,7 +1268,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor).</t>
+          <t>PASS — WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor) | 2026-08-15 re-verified live: home @graph carries WebSite + Person; Person has name/url/sameAs/jobTitle/worksFor — no missing fields | 2026-08-25 re-verified live: WebSite + Person @graph complete on /; Person carries name, url, sameAs, jobTitle, worksFor. | 2026-08-27 re-verified live: WebSite + Person @graph complete (name/url/sameAs/jobTitle/worksFor). | 2026-09-01 re-verified live: homepage @graph carries WebSite + Person; Person has name, url, sameAs, jobTitle, worksFor — zero required fields missing.</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1309,7 +1317,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description).</t>
+          <t>PASS — ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description) | 2026-08-15 re-verified live: about ProfilePage mainEntity Person complete — name/url/jobTitle/worksFor/sameAs/description all present | 2026-08-25 re-verified live: ProfilePage on /about/ with mainEntity @type Person carrying name, url, jobTitle, worksFor, sameAs, description. | 2026-08-27 re-verified live: ProfilePage mainEntity Person complete (name/url/jobTitle/worksFor/sameAs/description). | 2026-09-01 re-verified live: /about/ ProfilePage mainEntity is @type Person with name, url, jobTitle, worksFor, sameAs, description — zero missing.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1358,7 +1366,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one.</t>
+          <t>PASS — BlogPosting complete on all 16 (headline, description, datePublished, dateModified, author Person, publisher Organization+logo, mainEntityOfPage, image, url, inLanguage, wordCount); image == og:image exactly, no og-default drift | 2026-08-13 re-verified live: all 16 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount); zero og-default.png drift. | 2026-08-16 re-verified live: all 16 BlogPosting blocks re-verified live: every required field present (headline, description, datePublished, dateModified, author.@type=Person, publisher, mainEntityOfPage, image, url, inLanguage, wordCount) and JSON-LD image === og:image exactly, cache-bust included, on all 16. Zero og-default.png drift. | 2026-08-25 re-verified live: BlogPosting on all 16 articles; every required field present (headline, description, datePublished, dateModified, author.Person.name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero og-default.png regressions. | 2026-08-27 re-verified live: BlogPosting complete on all 16 — all 11 required fields, author.@type=Person, og:image == JSON-LD image, image == og-&lt;slug&gt;.png on every one. | 2026-09-01 re-verified live: all 17 BlogPosting blocks carry every required field (headline, description, datePublished, dateModified, author.@type=Person + name, publisher, mainEntityOfPage, image, url, inLanguage, wordCount). Zero on og-default.png.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1456,7 +1464,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml.</t>
+          <t>PASS — robots.txt Allow / + Sitemap → sitemap-index.xml | 2026-08-13 re-verified live: /robots.txt 200, Sitemap directive -&gt; https://imjustdex.com/sitemap-index.xml. | 2026-08-25 re-verified live: robots.txt = "User-agent: *\nAllow: /\n\nSitemap: https://imjustdex.com/sitemap-index.xml". /DESIGN-SYSTEM.md correctly 404s. | 2026-08-27 re-verified live: robots.txt Allow / + Sitemap → sitemap-index.xml. | 2026-09-01 re-verified live: robots.txt is 'User-agent: * / Allow: / / Sitemap: https://imjustdex.com/sitemap-index.xml'. /DESIGN-SYSTEM.md still 404s (the only thing keeping the doc unexposed).</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1505,7 +1513,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present.</t>
+          <t>PASS — sitemap-0.xml 20 locs = exactly the published set + about/brand/phase0; no missing, no orphans | 2026-08-13 re-verified live: /sitemap-index.xml -&gt; sitemap-0.xml; sitemap-0 lists 20 URLs covering all 16 articles + /, /about/, /brand/, /phase0/. Zero missing. | 2026-08-25 re-verified live: sitemap-index.xml references sitemap-0.xml; sitemap-0.xml carries exactly 20 locs = 16 articles + /, /about/, /brand/, /phase0/. The drafted essay is correctly absent. | 2026-08-27 re-verified live: sitemap-0.xml 20 locs; every homepage-linked route plus /about/ /brand/ /phase0/ present. | 2026-09-01 re-verified live: /sitemap-index.xml points to sitemap-0.xml; sitemap-0.xml holds exactly 21 URLs — the 17 live articles plus /, /about/, /brand/, /phase0/. Zero missing, zero extra. The drafted entry before-i-had-the-words is correctly absent.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1558,7 +1566,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one.</t>
+          <t>404 half PASS (noindex,nofollow live). Coming-soon half PENDING — no upcoming entry exists to render one | 2026-08-25: 404 half re-verified live (meta robots noindex,nofollow present, bespoke body served at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one. | 2026-09-01 404 half re-verified live (meta robots 'noindex, nofollow', bespoke body at HTTP 200). Coming-soon half still PENDING — no upcoming entry exists to render one.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -1709,7 +1717,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03.</t>
+          <t>PASS — Faith 13 / Identity 09 / Art 03, verified against frontmatter lanes; 16 articles | 2026-08-13 re-verified live: lane-index counts Faith 13 / Identity 09 / Art 03 — non-negative, zero-padded, and consistent with 16 essays counted per lane (15 .plate-lane chips + 1 .lead-badge-lane). | 2026-08-25 re-verified live: lane counts render Faith 13 / Identity 09 / Art 03 — matches the frontmatter tally across the 16 tracked essays exactly (multi-lane counted per lane). | 2026-08-27 re-verified live: lane counts Faith 13 / Identity 09 / Art 03. | 2026-09-01 re-verified live: lane-index reads Faith 14 / Identity 10 / Art 03 — non-negative integers summing to 27 across 17 essays (multi-lane counted per lane). Cross-checked against the filter: selecting Faith reveals exactly 14 articles.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -1762,7 +1770,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct.</t>
+          <t>PASS — live-verified 2026-08-10: Faith 13/13, Identity 9/9, Art 3/3 with zero non-matching plates in any filtered view; while filtered the .earlier-more-wrap computes display:none, 0 client rects, offsetHeight 0 (unreachable by mouse or keyboard). The ab07b15 fix holds in production. | 2026-08-16 re-verified live: all three lanes re-verified live: Faith 13, Identity 9, Art 3 — exactly matching the lane-index counts. Verified against the real filter key (data-lane, space-separated) rather than the visible chips: all 9 identity plates carry 'identity' in data-lane. While filtered, .earlier-more-wrap computes display:none with 0 client rects; clearing restores display:flex. | 2026-08-27 re-verified live: real pointer clicks: Faith 13, Identity 9, Art 3, re-click clears to the default 8; aria-pressed single-select correct. | 2026-09-01 re-verified live: .lane-cell[data-lane=faith] click sets aria-pressed=true and reveals exactly 14 articles; clicking again returns aria-pressed=false and the default 7-article view.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -1966,7 +1974,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track.</t>
+          <t>PASS — live-verified 2026-08-10: expand 8→16, collapse 16→8, aria-expanded false↔true and the button label track; collapse state survives a full filter cycle (clear restores the wrap to display:flex). | 2026-08-16 re-verified live: expand 8-&gt;16 and collapse 16-&gt;8 re-verified live; aria-expanded false&lt;-&gt;true and the label tracked ('View Earlier Essays — 8 more' &lt;-&gt; 'Show Less — showing all'); collapse state survived a full filter cycle. | 2026-08-27 re-verified live: real pointer clicks: 8→16→8, aria-expanded false↔true, label and count track. | 2026-09-01 re-verified live: toggle expands 10 hidden articles to 0 hidden, label 'View Earlier Essays — 10 more' -&gt; 'Show Less — showing all', aria-expanded false-&gt;true; collapse restores all three.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -2272,7 +2280,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16.</t>
+          <t>PASS — eyebrow lanes/tags + ' + ' separator, date, read time, h1, deck | 2026-08-27 re-verified live: eyebrow lanes/date/read-time render on all 16. | 2026-09-01 re-verified live on VOL 17 at 375px: eyebrow renders 4 lane/tag chips + date + read-time, all inside the frame post-F97.</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2378,7 +2386,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset.</t>
+          <t>PASS — bar width 0→249→698→1153px and aria-valuenow 0→30→69→100 across the scroll range. 2026-08-10 PM re-check: structural half re-verified (progress.js math recomputed by hand at 50% scroll = 51.5%; .article-body + .reading-progress present; role/aria-label/aria-valuemin/max initialized on load). Runtime paint not re-exercisable this run — the browser pane reports document.visibilityState 'hidden', so requestAnimationFrame never fires and the CSS width transition stays frozen at 0. Harness limitation, not a site regression. | 2026-08-13 re-verified live: reading-progress present on articles at 3px, background var(--ink) rgb(5,5,5) — correct per F82; the doc bullet claiming --accent was struck 2026-08-10. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The reading-progress bar is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2431,7 +2439,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset.</t>
+          <t>PASS — pill text tracks sections ('What the Fear Was Actually About' → 'A New Thing' → 'The Thirtieth'), opacity animates in. 2026-08-10 PM re-check: section collection re-verified live (5 .section-head h2 landmarks found on /words/send-someone-else/; the 40%-viewport rule resolves to the correct current section). Opacity fade not observable this run — same hidden-tab rAF/transition suspension as F35. | 2026-08-27 NOT re-verified — rotation gap, not a failure. The section-indicator pill is scroll-driven and the browser pane would not scroll this run (window.scrollTo, scrollingElement.scrollTop, Page_Down x6 and the pointer scroll action all left scrollY at 0-2 on an 11,937px article; the pointer scroll action timed out with 'Browser pane is currently hidden'). Source unchanged since the last PASS, so the row keeps its prior result rather than being reset. | 2026-09-01 NOT TESTABLE this run — rotation gap, prior result retained. The browser pane went hidden: the pointer scroll timed out with 'Browser pane is currently hidden' and window.scrollTo / scrollingElement.scrollTop both left scrollY at 0 against a 10905px document. The .reading-progress element itself is present and correctly wired (role=progressbar, aria-valuenow=0, width 0% at scrollY 0). Neither PASS nor FAIL recorded, per the documented harness antipattern.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -2949,7 +2957,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future.</t>
+          <t>PENDING — all 16 entries are status published with past dates, so isUpcomingData() is false everywhere and no coming-soon page renders | 2026-08-25: still PENDING for the same structural reason — all 16 built entries are status:published with past dates. NOTE: an untracked draft (src/content/words/before-i-had-the-words.mdx, status:"drafted", publishedDate 2026-08-07) sits in Dexter's working tree. It is correctly excluded from the build (19 pages, 16 articles) and does not exercise this path either, since its date is in the past, not the future. | 2026-09-01 still PENDING. The untracked draft in Dexter's working tree (src/content/words/before-i-had-the-words.mdx, status 'drafted', publishedDate 2026-08-07) is correctly excluded from the build (20 pages, 17 articles) but does NOT exercise this path — its date is in the past and its status is 'drafted', not an upcoming publish. Left untouched.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -3002,7 +3010,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render.</t>
+          <t>PASS — about content + ProfilePage render | 2026-08-27 re-verified live: about content + ProfilePage render. | 2026-09-01 re-verified live: /about/ 200 in 0.75s, single h1, all four landmarks, 0 contrast failures across 24 measured elements.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -3104,7 +3112,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1.</t>
+          <t>PASS — bespoke notfound-plate, 200 on /404, noindex+nofollow, /* fallback 404s unmatched routes | 2026-08-27 re-verified live: bespoke notfound-plate, 200 on /404, noindex+nofollow, single h1. | 2026-09-01 re-verified live: /404 returns HTTP 200 with the bespoke 'Nothing to Document Here' body, meta robots noindex,nofollow, single h1, all four landmarks, 0 contrast failures across 16 elements.</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -3157,7 +3165,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage.</t>
+          <t>PASS — Atom 16 entries = 16 published; namespace + entries valid | 2026-08-13 re-verified live: /feed.xml 200, Atom namespace, 16 &lt;entry&gt; elements — exactly matching the 16 articles on the homepage, zero set difference either direction. | 2026-08-16 re-verified live: /feed.xml 200 with 16 &lt;entry&gt; elements; set-compared against the 16 article links on the live homepage — zero difference in either direction. | 2026-08-25 re-verified live: /feed.xml 200, 16 &lt;entry&gt; elements matching the 16 published articles exactly — no gaps, no extras. | 2026-08-27 re-verified live: Atom 16 entries == 16 published on the homepage. | 2026-09-01 re-verified live: /feed.xml 200, 17 entries — exactly matching the 17 articles on the homepage cascade. No feed-only or home-only slugs.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
@@ -3210,7 +3218,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present.</t>
+          <t>PASS — feed.xsl 200 and &lt;?xml-stylesheet?&gt; PI present | 2026-08-13 re-verified live: /feed.xsl 200 and referenced via &lt;?xml-stylesheet?&gt; in the feed prolog. | 2026-08-25 re-verified live: /feed.xsl 200 and feed.xml carries &lt;?xml-stylesheet href="/feed.xsl"?&gt;. | 2026-08-27 re-verified live: feed.xsl 200 and the &lt;?xml-stylesheet?&gt; PI is present. | 2026-09-01 re-verified live: /feed.xml carries the &lt;?xml-stylesheet?&gt; reference and /feed.xsl returns 200.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3263,7 +3271,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets.</t>
+          <t>PASS — 5 anchor links, all resolve to real targets | 2026-08-27 re-verified live: 5 anchor links on /phase0/, all resolve to real targets. | 2026-09-01 re-verified live: /phase0/ 200 in 0.41s, single h1, no skipped heading levels across a 22-heading tree, 0 contrast failures across 106 measured elements.</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
@@ -3422,7 +3430,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/ serves plates.css?v=phase15, matching every other surface; no second year-long cache entry. | 2026-09-01 re-verified live: /brand/ 200, single h1, no skipped heading levels, 0 contrast failures across 800 measured elements in dark mode.</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -3899,7 +3907,7 @@
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical.</t>
+          <t>PASS — /about, /phase0 and all 16 /words/&lt;slug&gt; → single 301 to trailing-slash canonical | 2026-08-13 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200; /sitemap.xml correctly 404 post-cutover. | 2026-08-16 re-verified live: /about -&gt; 301 -&gt; /about/ -&gt; 200 and /words/the-stone -&gt; 301 -&gt; /words/the-stone/ re-verified live; /sitemap.xml correctly 404 post-cutover; /words -&gt; 301 home; /opsmeeting -&gt; 301 home. | 2026-08-25 re-verified live: /about, /brand, /phase0 and /words/the-stone each return a single 301 to the trailing-slash form, which returns 200. No loops. | 2026-08-27 re-verified live: /about and /words/the-stone → single 301 to the trailing-slash canonical. | 2026-09-01 re-verified live: /about -&gt; 301 -&gt; https://imjustdex.com/about/ -&gt; 200.</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
@@ -4058,7 +4066,7 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function.</t>
+          <t>PASS — /api/subscribe rewrite reaches the function (405 on GET, 400/200 on POST) | 2026-08-13 re-verified live: /api/subscribe rewrite reached the Netlify function and returned a Mailchimp success body. | 2026-08-25 re-verified live: /api/subscribe rewrite to the Netlify function verified by the live smoke POST. | 2026-08-27 re-verified live: /api/subscribe rewrite reaches the function. | 2026-09-01 re-verified live: POST to /api/subscribe rewrote to the Netlify function and returned 200.</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr"/>
@@ -4164,7 +4172,7 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article.</t>
+          <t>PASS — CSP present and strict on every page; per-route /brand/ + /feed.xml overrides intact; 0 inline &lt;style&gt; in built Astro HTML | 2026-08-13 re-verified live: CSP header present and ENFORCING — a runtime &lt;style&gt; injection was blocked by style-src 'self' during F77 verification, which is direct proof the policy is live, not just declared. Per-route /brand/ and /feed.xml relaxations by design. | 2026-08-16 re-verified live: CSP present and strict on every page type; /brand/ and /feed.xml keep their by-design style-src 'unsafe-inline' relaxation. Zero inline &lt;style&gt; blocks in any built Astro page (home 0, article 0, about 0, phase0 0). Policy proven live again this run — a &lt;style&gt; injection was blocked, while CSSOM mutation of the already-loaded sheet succeeded, which is the documented distinction. | 2026-08-25 re-verified live: CSP present on every route and empirically ENFORCED — an injected inline &lt;style&gt; during this run was blocked by style-src 'self' and logged as the only console error of the whole scrub. Per-route relaxation for /brand/ (style-src adds 'unsafe-inline') confirmed by design. Zero inline &lt;style&gt; blocks in any built page. | 2026-08-27 re-verified live: CSP present and strict on / and on an article. | 2026-09-01 re-verified live: CSP present and identical on / and /words/&lt;slug&gt;/ — default-src 'self'; script-src 'self'; style-src 'self'; img-src 'self' data: https:; font-src 'self'; connect-src 'self'; frame-ancestors 'none'; base-uri 'self'; form-action 'self'; object-src 'none'; upgrade-insecure-requests. Zero inline &lt;style&gt; blocks in any built or served page (CSP would block them).</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
@@ -4217,7 +4225,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present.</t>
+          <t>PASS — X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy, Permissions-Policy, COOP, CORP on all 21 routes | 2026-08-13 re-verified live: all 5 security headers present on all 6 page types (home, article, about, brand, phase0, 404, feed): X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present. | 2026-08-16 re-verified live: all security headers re-verified live on home/article/brand/404/feed: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000 includeSubDomains preload, CSP, Referrer-Policy strict-origin-when-cross-origin, Permissions-Policy, COOP same-origin, CORP same-origin. | 2026-08-25 re-verified live: all five headers present on / and on an article: X-Frame-Options DENY, X-Content-Type-Options nosniff, HSTS max-age=31536000; includeSubDomains; preload, CSP, Referrer-Policy strict-origin-when-cross-origin. Permissions-Policy also present on /. | 2026-08-27 re-verified live: X-Frame DENY, nosniff, HSTS max-age=31536000 includeSubDomains preload, Referrer-Policy all present. | 2026-09-01 re-verified live: X-Frame-Options DENY, X-Content-Type-Options nosniff, Strict-Transport-Security max-age=31536000; includeSubDomains; preload, Referrer-Policy strict-origin-when-cross-origin — all present on / and on an article.</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr"/>
@@ -4270,7 +4278,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable.</t>
+          <t>PASS — live-verified 2026-08-10: /brand/brand.css?v=brand5 and /img/* both return public,max-age=31536000,immutable; HTML remains public,max-age=0,must-revalidate. | 2026-08-13 re-verified live: versioned assets (/css, /js, /img) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-16 re-verified live: versioned assets (/css, /js, /img, /fonts) all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift. | 2026-08-25 re-verified live: versioned CSS, fonts and images all serve public,max-age=31536000,immutable; HTML serves public,max-age=0,must-revalidate. No drift on either tier. | 2026-08-27 re-verified live: HTML no-cache/must-revalidate; /css/*?v= and /img/* both public,max-age=31536000,immutable. | 2026-09-01 re-verified live: /css/tokens.css?v=phase24 and /fonts/Anton-Regular.woff2 both return public,max-age=31536000,immutable; HTML returns public,max-age=0,must-revalidate. No drift on either pattern.</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
@@ -4376,7 +4384,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Medium (2026-08-27) — the scheduled run did not fire today. GitHub Actions shows 'Daily rebuild' completing every day 2026-08-19 through 2026-08-26 at 05:35-05:47Z; there is no run for 2026-08-27, checked at 14:06Z — 9h past the 05:05 UTC cron. Workflow state is 'active' and the YAML is unchanged and valid, so this is GitHub dropping/delaying the schedule, not a repo defect. Netlify's newest ready deploy is 2026-08-26T05:43Z (commit_ref b64a39b == GitHub main HEAD). Live impact today: none — zero date-gated essays are pending (F30 correctly absent), so the rebuild would have produced byte-identical output. It matters the day an essay is scheduled. | CORRECTION 2026-08-28. Yesterday's conclusion was WRONG IN ITS CAUSE. I reported at 14:06Z that no run existed for 2026-08-27 and inferred GitHub had dropped the schedule. The run did happen — at 16:23:33Z, about 11.3 hours after the 05:05Z cron and about two hours after I looked. Today's fired at 17:21:17Z, about 12.3 hours late. So the real finding is not a dropped run but a DRIFTED one: the workflow moved from a steady 05:35-05:47Z window (2026-08-19 through 08-26) to 16:23-17:21Z on the two days since. Still open, still GitHub-side, and still worth knowing — a date-gated essay would go live roughly twelve hours after its intended 00:00 CST rather than roughly forty minutes after. The measurement was sound; the inference from a single missing data point was not, and 'checked once, concluded never' is the antipattern to carry forward.</t>
+          <t>ISSUE/Medium (2026-08-27) — the scheduled run did not fire today. GitHub Actions shows 'Daily rebuild' completing every day 2026-08-19 through 2026-08-26 at 05:35-05:47Z; there is no run for 2026-08-27, checked at 14:06Z — 9h past the 05:05 UTC cron. Workflow state is 'active' and the YAML is unchanged and valid, so this is GitHub dropping/delaying the schedule, not a repo defect. Netlify's newest ready deploy is 2026-08-26T05:43Z (commit_ref b64a39b == GitHub main HEAD). Live impact today: none — zero date-gated essays are pending (F30 correctly absent), so the rebuild would have produced byte-identical output. It matters the day an essay is scheduled. | CORRECTION 2026-08-28. Yesterday's conclusion was WRONG IN ITS CAUSE. I reported at 14:06Z that no run existed for 2026-08-27 and inferred GitHub had dropped the schedule. The run did happen — at 16:23:33Z, about 11.3 hours after the 05:05Z cron and about two hours after I looked. Today's fired at 17:21:17Z, about 12.3 hours late. So the real finding is not a dropped run but a DRIFTED one: the workflow moved from a steady 05:35-05:47Z window (2026-08-19 through 08-26) to 16:23-17:21Z on the two days since. Still open, still GitHub-side, and still worth knowing — a date-gated essay would go live roughly twelve hours after its intended 00:00 CST rather than roughly forty minutes after. The measurement was sound; the inference from a single missing data point was not, and 'checked once, concluded never' is the antipattern to carry forward. | 2026-09-01 drift CONFIRMED as a persistent pattern, not a one-off. Cron is '5 5 * * *' (05:05 UTC). Five consecutive hook-triggered deploys read from the Netlify API: 08-28 17:21Z, 08-29 11:35Z, 08-30 10:26Z, 08-31 11:31Z, 09-01 09:57Z. Today's fired 4h52m late; the window across five days is +4h52m to +12h16m. It fires EVERY day (never missed), so this is GitHub Actions scheduled-workflow queue latency, not a broken workflow. BLOCKED for auto-fix: the repo-side cron is already correct and editing it cannot shorten GitHub's queue; the only real remedy (move the trigger to a Netlify scheduled function) is a Netlify-dashboard change outside the repo. NEEDS DEXTER if publish-hour precision ever has to be guaranteed.</t>
         </is>
       </c>
       <c r="I76" s="7" t="inlineStr">
@@ -4433,7 +4441,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200.</t>
+          <t>PASS — scripts/og-plate.mjs present; all 19 OG plates render and 200 | 2026-08-27 re-verified live: all 21 OG plates 200. | 2026-09-01 re-verified live: every one of the 17 per-article OG plates resolves 200 at its cache-busted path; none falls back to og-default.png.</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>
@@ -4486,7 +4494,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets.</t>
+          <t>PASS — @media (prefers-reduced-motion: reduce) block in tokens.css (loads on every page) | 2026-08-13 re-verified live: verified in the DEPLOYED sheet, not just source: tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, *::before, *::after with !important, plus scroll-behavior auto. Catches all 29 transitioned elements on the homepage. | 2026-08-16 re-verified live: re-verified in the LOADED CSSOM (not source): tokens.css?v=phase23 carries @media (prefers-reduced-motion: reduce) zeroing transition-duration and animation-duration on *, ::before, ::after with !important plus scroll-behavior auto — catching all 8 transitioned elements on the article page. | 2026-08-25 re-verified live: tokens.css:584 zeroes transition-duration and animation-duration on *, ::before and ::after under prefers-reduced-motion: reduce and sets scroll-behavior auto; home-augment.css:1012 adds the targeted transition:none block. Both present in the served sheets. | 2026-08-27 re-verified live: @media (prefers-reduced-motion: reduce) block present in the loaded stylesheets. | 2026-09-01 SOURCE-VERIFIED only: tokens.css?v=phase24 carries a blanket @media (prefers-reduced-motion: reduce) block setting transition-duration and animation-duration to 0s !important on *, *::before and *::after, plus scroll-behavior: auto on html; home-augment.css adds two scoped blocks. The !important universal selector is cascade-proof, so the rule cannot be defeated downstream. NOT re-verified in the browser: this harness cannot emulate the prefers-reduced-motion media query. Prior live PASS retained.</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
@@ -4539,7 +4547,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent.</t>
+          <t>PASS (closed live 2026-08-10) — was ISSUE/High: .subscribe-manifesto .sm-submit (homepage + /brand/ subscribe submit) had base and :hover styling but NO :focus-visible rule, so the site's primary conversion control showed no focus indicator for keyboard users (WCAG 2.4.7 AA). Every sibling control was covered — .sm-input directly above it had the rule, and .sm-submit was even named in home-augment.css's prefers-reduced-motion block — so it was an omission, not a decision. Missed by prior runs because F76 was tested at sheet level (':focus-visible present in all 8 stylesheets') rather than per control. Fixed and deployed same day; see p3/p4. | 2026-08-13 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to a footer link that matched ':focus-visible' and computed outline 'solid 2px rgb(204, 0, 0)' at offset 2px. | 2026-08-16 re-verified live: re-verified live by REAL keyboard input (not JS .focus(), which cannot trigger :focus-visible): pressing Tab moved focus to SUMMARY.study-note-trigger, which matched ':focus-visible' and computed outline 'rgb(204, 0, 0) solid 2px' at offset -2px. | 2026-08-25 re-verified live: re-verified under REAL keyboard input: tabbing to .study-note-trigger on an article paints outline solid 2px rgb(204,0,0) (--focus-ring) at -2px offset. NOTE for future runs: a programmatic element.focus() does NOT satisfy :focus-visible in Chrome and will report outline:none across the board — a false positive this run initially produced. | 2026-08-27 re-verified live: focus ring under REAL Tab (not element.focus()): outline rgb(204,0,0) solid 2px = --accent. | 2026-09-01 re-verified live under REAL Tab presses (never element.focus()): .brand-block, .mode-toggle, .issue-standfirst and .hero-link each match :focus-visible and paint outline rgb(204,0,0) solid 2px, matching --focus-ring #c00.</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4596,7 +4604,7 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression.</t>
+          <t>PASS (closed live 2026-08-13) — was ISSUE/High (2026-08-13) — .latest-tag (the red 'Latest' chip in the homepage standfirst bar) pairs `background: var(--accent)` with `color: var(--bg)`. In light mode that is cream on #c00 = 5.17:1 and passes. In dark mode --bg flips to #060606 and the same chip computes 3.44:1 at 11.52px/700 — under the 4.5:1 AA floor for small text (WCAG 1.4.3). Measured three times on settled live loads. The #c00/#060606 pair is sanctioned by the Phase 4.1 accent doctrine (DESIGN-SYSTEM.md:102) only for NON-text contrast at the 3:1 floor; this is a text use of it. Missed by prior runs because F77 sampled palette-level token pairs (body/muted/faint/accent text), not the one control that puts small text ON the accent fill — the same sheet-level vs per-control gap that hid F76. All other sampled combinations still pass: 33 distinct fg/bg/size combos in dark, 33 in light, this was the only failure. | 2026-08-16 re-verified live: full-page compositor sweep across home (dark 92 elements / light 88), article (70), about (15), phase0 (84), brand and 404. Two light-mode 'failures' on .plate-image plates (h2.plate-title.inverse and p.plate-deck, both 1.06:1) were investigated and DISMISSED as false positives: those plates carry an ::after `linear-gradient(to top, rgba(0,0,0,.78) ...)` scrim, so the white text sits on a dark overlay, not the cream plate colour the compositor resolved — confirmed visually in a light-mode screenshot. Two compounding methodology bugs were behind the false read and are now fixed in the sweep: (a) the compositor walked background-COLOR only and ignored pseudo-element layers, (b) selector-level dedupe merged image and non-image plates under the same class string, so a passing element inherited a failing element's number. Lesson is the same shape as F84's: resolve the PAINTED surface, never infer it from an ancestor's declarations. | 2026-08-25 re-verified live: .latest-tag on the live homepage in dark mode measures 5.17:1 (rgb(243,240,232) on rgb(204,0,0)) — the F77 fix still holds, no regression. | 2026-09-01 re-verified live with a full ancestor-stack compositing probe (semi-transparent layers composited down to the first opaque one; .plate-image plates and aria-hidden decoration excluded per the documented antipatterns): 0 WCAG AA failures across ~1050 measured text elements — homepage light (0/70+), homepage dark (0/70), article dark at 375px (0/86), /about/ (0/24), /404 (0/16), /phase0/ (0/106), /brand/ (0/800).</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -4653,7 +4661,7 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes.</t>
+          <t>PASS — single h1 and zero skipped heading levels on all 21 pages; header/main/footer/nav present; zero &lt;img&gt; without alt | 2026-08-13 re-verified live: home and article both single-h1, zero skipped heading levels (home H1 then 17x H2; article H1,H2,H2,H2,H2,H2), header/main/footer/nav all present. Zero images missing alt. | 2026-08-16 re-verified live: single &lt;h1&gt; and zero skipped heading levels across all 21 live pages; header/main/footer/nav present on every page type; zero &lt;img&gt; without an alt attribute. | 2026-08-25 re-verified live: header/main/footer/nav present on every page type; exactly one &lt;h1&gt; per page across all 20 routes; zero skipped heading levels; zero &lt;img&gt; without alt. | 2026-08-27 re-verified live: single h1 and zero skipped heading levels across all 21 routes. | 2026-09-01 re-verified live: header/main/footer/nav present on every route; exactly one h1 per page; no skipped heading levels anywhere, including /phase0/'s 22-heading tree.</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
@@ -4759,7 +4767,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200.</t>
+          <t>PASS — parity 16/16 verified live; every /words/&lt;slug&gt; returns a single 301 to its trailing-slash canonical; no orphan rules | 2026-08-13 re-verified live: all 16 /words/&lt;slug&gt; (no trailing slash) return 301; all 16 /words/&lt;slug&gt;/ return 200 in 0.31-0.45s. | 2026-08-25 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200. | 2026-09-01 re-verified live: /words/the-stone -&gt; 301 -&gt; /words/the-stone/ -&gt; 200.</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr"/>
@@ -5431,7 +5439,7 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4.</t>
+          <t>ISSUE/Low (2026-08-27) — the click handler rewrote the label and the count but never touched the glyph. Live on b64a39b the expanded state reads 'Show Less — showing all ↓': the arrow still points down, i.e. 'more below', while the button's own words say it will collapse. The glyph carries aria-hidden="true" so nothing is exposed to assistive tech — this is a purely visual affordance contradiction, which is why it survived every prior scrub. | RESOLVED LIVE 2026-08-27 — see p4. | 2026-09-01 re-verified live: .btn-glyph tracks the button state — down-arrow collapsed, up-arrow expanded, and back.</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -5655,7 +5663,7 @@
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay.</t>
+          <t>PASS (2026-08-31, live on 13b631c then 83c2137) — POST-gate half verified live end to end: article 200 with 55 paragraphs and zero coming-soon markers; present in sitemap-0.xml, feed.xml and the homepage cascade (latest strip, lead plate, 'Week of August 31, 2026'); 'Send Someone Else' renders 0 .article-nav-ghost, i.e. the ghost treatment retired itself on go-live exactly as designed. OG plate 1200x630 (1.905), reads VOL 17 matching the essay's own number, title clears Anton's caps on the .92 leading from 9301d61. Metadata complete (description, og:title/image/image:alt/type, twitter:summary_large_image, canonical). Redate to Aug 31 propagated to every surface: JSON-LD datePublished 2026-08-31T12:00:00-05:00, Atom &lt;published&gt; 2026-08-31T17:00:00Z, homepage &lt;time datetime="2026-08-31"&gt;, zero 'Aug 30' anywhere live. Contrast 87 elements / 0 failures in BOTH modes (dark floor 5.13:1, light 4.67:1). Single h1, h1-&gt;h2 with no skipped level, skip link takes first Tab with a visible ring, 0 unnamed interactive elements, 0 console errors. || PRE-gate half NOT verified in production — see F93/F94: the release sat unpushed from Aug 29 until after the Aug 30 noon gate, so the Coming-Soon route never rendered on the live site for this essay. | 2026-09-01 re-verified live: VOL 17 present and correct across article (200), homepage lead plate, feed (17/17), sitemap and OG plate; article:published_time 2026-08-31 matches the homepage plate's &lt;time datetime&gt;.</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr"/>
@@ -5705,7 +5713,7 @@
       </c>
       <c r="I100" s="6" t="inlineStr">
         <is>
-          <t>High (fixed)</t>
+          <t>High (closed live)</t>
         </is>
       </c>
       <c r="J100" s="4" t="inlineStr">
@@ -5715,7 +5723,7 @@
       </c>
       <c r="K100" s="6" t="inlineStr">
         <is>
-          <t>PASS (verified against build) — 2026-08-31 on a clean `npm run build` served from dist at 375x812. ALL 18 pages carrying .article-eyebrow re-tested, not a sample: about (1 chip), gumbo/job/next-verse/price-of-sunday (3), gloria/outsourced-faith/pulpit/reckonings/show-me-your-glory/some/the-nets/the-stone (4), music-that-raised-me/not-the-same-as-alive/send-someone-else/should-have-killed-it (5), the-weight-of-my-no (6). Every page: flex-wrap resolves `wrap`, eyebrow overflow 0px, every chip fully visible, document horizontal scroll 0. Regression check at a true emulated 1280px desktop: local build and live production are identical (flex-wrap nowrap, overflow 0) — the change is mobile-only and touches no desktop layout. Built pages confirmed serving article.css?v=phase37.</t>
+          <t>PASS (verified against build) — 2026-08-31 on a clean `npm run build` served from dist at 375x812. ALL 18 pages carrying .article-eyebrow re-tested, not a sample: about (1 chip), gumbo/job/next-verse/price-of-sunday (3), gloria/outsourced-faith/pulpit/reckonings/show-me-your-glory/some/the-nets/the-stone (4), music-that-raised-me/not-the-same-as-alive/send-someone-else/should-have-killed-it (5), the-weight-of-my-no (6). Every page: flex-wrap resolves `wrap`, eyebrow overflow 0px, every chip fully visible, document horizontal scroll 0. Regression check at a true emulated 1280px desktop: local build and live production are identical (flex-wrap nowrap, overflow 0) — the change is mobile-only and touches no desktop layout. Built pages confirmed serving article.css?v=phase37. | 2026-09-01 LIVE-VERIFIED on production (deploy 885930e): /words/the-weight-of-my-no/ at an emulated 375x812 — computed flex-wrap: wrap, eyebrow scrollWidth == clientWidth (301px, 0px overflow), rail lays out on two rows at 68px tall, and all 6 children render inside the frame with the read-time chip ('8 min', right edge 277px) fully visible. documentElement.scrollWidth == clientWidth == 375 — no horizontal document overflow. article.css?v=phase37 confirmed serving the wrap rule. F97 CLOSED LIVE.</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5855,7 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">

</xml_diff>